<commit_message>
TigerGraph HA node-failure testing: cluster, test suite, and report
Deploy a 3-node TigerGraph 4.1.4 cluster with high availability (replication
factor 2) and test its behaviour under node failures.

- 17 test cases: service health, GSQL query combinations, CSV loading job,
  six node-failure modes, write durability, negative and boundary scenarios
- MTTR measured with a 250ms availability probe from a surviving node; each
  failure scenario repeated 3x, medians reported with min-max spread
- Docs: test report (md/pdf), test plan and traceability matrix (xlsx/pdf),
  execution results, findings, screenshots, per-test logs
- Reproducible: docker compose + install script + uv run pytest
</commit_message>
<xml_diff>
--- a/docs/TestExecutionReport.xlsx
+++ b/docs/TestExecutionReport.xlsx
@@ -695,22 +695,22 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>42.56</v>
+        <v>22.88</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>43.82</v>
+        <v>23.86</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>85.23%</t>
+          <t>94.89%</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Recovered via replica failover.</t>
+          <t>Recovered via replica failover. Median of 3 runs (MTTR 23.53-30.5 s).</t>
         </is>
       </c>
     </row>
@@ -736,22 +736,22 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>22.89</v>
+        <v>22.95</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>23.64</v>
+        <v>23.68</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>94.96%</t>
+          <t>94.89%</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Recovered via replica failover.</t>
+          <t>Recovered via replica failover. Median of 3 runs (MTTR 23.67-23.95 s).</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Zero downtime - replica served throughout.</t>
+          <t>Zero downtime - replica served throughout. Median of 3 runs.</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Zero downtime - replica served throughout.</t>
+          <t>Zero downtime - replica served throughout. Median of 3 runs.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Zero downtime - replica served throughout.</t>
+          <t>Zero downtime - replica served throughout. Median of 3 runs.</t>
         </is>
       </c>
     </row>
@@ -888,22 +888,22 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.06</v>
+        <v>0.45</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>42.53</v>
+        <v>22.91</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>43.69</v>
+        <v>23.91</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>83.75%</t>
+          <t>94.89%</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Recovered via replica failover.</t>
+          <t>Recovered via replica failover. Median of 3 runs (MTTR 23.88-43.97 s).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add bug reports with RCA, config-change test, and execution notes
- findings/: 4 bug reports with root-cause analysis (BUG-001..004, .md + .docx)
- tests/test_config_change.py (TC-CFG-001): change a service config via
  gadmin config set -> apply -> restart all; verify the value applies and all
  services return Online (RESTPP query-timeout var; reverted after)
- cluster.py: config_get/set/apply + restart_all helpers
- docs: REPORT/README to 18 cases; add bugs section, execution-model note
  (suite runs sequentially - failure tests share one cluster); regenerate
  TestPlan / TraceabilityMatrix / ExecutionReport / PDFs
- screenshots/SS-13: config-change + restart evidence
- stop tracking internal notes file
</commit_message>
<xml_diff>
--- a/docs/TestExecutionReport.xlsx
+++ b/docs/TestExecutionReport.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1070,6 +1070,37 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFG-001</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Configuration change: set a service config variable, apply and restart all; the value takes effect and all services return Online.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Config change applied after restart; all services returned Online (reverted after).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>